<commit_message>
Fix GitHub Actions workflows with legacy peer deps and resilient driver execution
</commit_message>
<xml_diff>
--- a/selenium-tests/selenium_test_report.xlsx
+++ b/selenium-tests/selenium_test_report.xlsx
@@ -17,7 +17,7 @@
     <t>🏥 HealthGenie AI - Web Frontend Selenium E2E Automation Report</t>
   </si>
   <si>
-    <t>Execution Date: 19/8/2026, 5:52:15 pm | Target Environment: http://localhost:5173 | Suite: Login &amp; Auth E2E</t>
+    <t>Execution Date: 19/8/2026, 6:09:43 pm | Target Environment: http://localhost:5173 | Suite: Login &amp; Auth E2E</t>
   </si>
   <si>
     <t>TOTAL TEST CASES</t>
@@ -182,7 +182,7 @@
     <t>CRITICAL</t>
   </si>
   <si>
-    <t>2026-08-19T12:22:15.797Z</t>
+    <t>2026-08-19T12:39:43.618Z</t>
   </si>
   <si>
     <t>TC-LOG-002</t>
@@ -209,7 +209,7 @@
     <t>HIGH</t>
   </si>
   <si>
-    <t>2026-08-19T12:22:15.798Z</t>
+    <t>2026-08-19T12:39:43.619Z</t>
   </si>
   <si>
     <t>TC-LOG-003</t>

</xml_diff>